<commit_message>
Parent Portal fully editable, Friday 9 AM lunch deadline, Miss Dove K3 Teacher, Monday homeroom lunch emails
- content/parents.json now holds the whole Parent Portal page (welcome text, every section's
  heading, rich text, links and PDFs, order); the office edits it in Pages CMS. Replaces
  content/documents.json. Section text is cleaned to simple formatting in build.py.
- Lunch order deadline defaults to 9:00 AM on the Friday before the week; the office can still
  type a different one.
- Staff and preschool pages: Natalie Dove is K3 Teacher.
- Lunch service: Mondays 7 AM Eastern, one email per homeroom teacher listing their students
  with hot lunch that week, Cc the office. Teachers come from a new Teachers tab in the
  workbook; the service adds Teachers and a live Homerooms tab if missing. Test workflow added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E7XcgKCmGLaKn6KwAGBL3a
</commit_message>
<xml_diff>
--- a/worker/Hot Lunch Orders.xlsx
+++ b/worker/Hot Lunch Orders.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kitchen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teachers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kitchen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -91,10 +92,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -639,6 +640,242 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Teacher</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Homeroom teacher for each grade. Type each teacher's email in column C. Keep the Grade column as it is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Preschool (K3)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Miss Dove</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Preschool (K4)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mrs. Febo</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Kindergarten (K5)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ms. Schmidley</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1st Grade</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Miss Ryans</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2nd Grade</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ms. Raymond</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3rd Grade</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mrs. Lundberg</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4th Grade</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mrs. Kirby</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5th Grade</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mrs. Baumgartner</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6th Grade</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mrs. Baumgartner</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>7th Grade</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mr. Napierala</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8th Grade</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mr. Napierala</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>9th Grade</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mr. Damm</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10th Grade</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mr. Damm</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>11th Grade</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mr. Greene</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12th Grade</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mr. Greene</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -650,23 +887,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Hot lunch counts</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Week of (Monday)</t>
         </is>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="6">
         <f>MAX(Orders[Week of])</f>
         <v/>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Shows the latest week. Type another Monday's date here to see that week.</t>
         </is>
@@ -815,12 +1052,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Week total</t>
         </is>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <f>SUM(E6:E10)</f>
         <v/>
       </c>
@@ -841,13 +1078,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -887,15 +1124,29 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
+          <t>Teachers: the Teachers tab lists each grade's homeroom teacher and email. Every Monday at 7:00 AM each teacher gets an email (Cc the office) listing their students with hot lunch that week. Update it each school year; a grade with no email gets no list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Homerooms: the Homerooms tab shows the same lists for this week, youngest grade first. The order service adds this tab by itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
           <t>Changes by phone: remove an X (or type X) under a day and the totals update. To cancel a whole order, delete the student's row. Use Notes for anything worth remembering.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Please don't rename this file, the Orders tab, the Orders table or its column headings, and don't move the file out of the OneDrive's main folder. The website needs them to add orders.</t>
         </is>

</xml_diff>